<commit_message>
Blocco 1 (collazione con la Rete): 9 portali della memoria annotati
Verifica per collazione con la Rete degli archivi per non dimenticare e riscontro
esterno. 6 confermati (verde): SIUSA, Mappe di Memoria, archivio900.it, Archivio di
Stato di Milano (fondo Piazza Fontana/Salvini), Archivio storico Corriere della Sera,
ArchivioAntimafia. 3 parziali (giallo): fontitaliarepubblicana.it (dominio da
riscontrare vs portalefontirepubblicaitaliana.cnr.it) e la duplicazione righe 14=15
(Associazione familiari Bologna = stragi.it, da sciogliere per §8.4). Annotazioni
in col. J/K/L con i colori del foglio; nomi propri disponibili registrati (es. giudice
Guido Salvini).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
+++ b/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -152,6 +152,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -6083,11 +6086,19 @@
       <c r="I11" s="3" t="inlineStr"/>
       <c r="J11" s="8" t="inlineStr">
         <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr"/>
-      <c r="L11" s="8" t="inlineStr"/>
+          <t>PARZIALE — l'ente esiste (Portale delle fonti per la storia della Repubblica italiana, infrastruttura del CNR, accesso unico a fonti dal 1946 [A]), ma il DOMINIO va accertato: le fonti danno il portale come portalefontirepubblicaitaliana.cnr.it, non fontitaliarepubblicana.it [B]. Da confermare che il dominio del repertorio risolva o rediriga.</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>COLLAZIONE RETE 6.8.2026: portalefontirepubblicaitaliana.cnr.it (CNR), Istituto Sturzo, storiadigitale.it; collegato al Centro Flamigni. DOMINIO DA RISCONTRARE.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -6123,13 +6134,21 @@
       <c r="G12" s="3" t="inlineStr"/>
       <c r="H12" s="3" t="inlineStr"/>
       <c r="I12" s="3" t="inlineStr"/>
-      <c r="J12" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K12" s="8" t="inlineStr"/>
-      <c r="L12" s="8" t="inlineStr"/>
+      <c r="J12" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — SIUSA, Sistema Informativo Unificato per le Soprintendenze Archivistiche (DG Archivi/ICAR con la Scuola Normale di Pisa): descrive il patrimonio archivistico non statale, pubblico e privato, conservato fuori dagli Archivi di Stato; soggetti produttori, conservatori e strumenti di ricerca [A].</t>
+        </is>
+      </c>
+      <c r="K12" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L12" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE RETE 6.8.2026: icar.cultura.gov.it, siusa-archivi.cultura.gov.it; dal 2011 esporta al Sistema Archivistico Nazionale (SAN). Ente confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -6217,11 +6236,19 @@
       <c r="I14" s="3" t="inlineStr"/>
       <c r="J14" s="8" t="inlineStr">
         <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr"/>
-      <c r="L14" s="8" t="inlineStr"/>
+          <t>CONFERMATO come ente, MA DUPLICATO DELLA RIGA 15: l'Associazione familiari delle vittime della strage di Bologna del 2.8.1980 È il soggetto titolare di stragi.it (riga 15) [A]. Duplicazione fra voci da sciogliere (§8.4); tenuta in sospeso finché non si decide quale conservare e fondere.</t>
+        </is>
+      </c>
+      <c r="K14" s="8" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L14" s="8" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: stragi.it, memoria.cultura.gov.it. STESSA ENTITÀ della riga 15.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -6259,11 +6286,19 @@
       <c r="I15" s="3" t="inlineStr"/>
       <c r="J15" s="8" t="inlineStr">
         <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr"/>
-      <c r="L15" s="8" t="inlineStr"/>
+          <t>CONFERMATO — stragi.it è il sito dell'Associazione familiari vittime strage Bologna 2.8.1980; archivio consultabile di foto, video, audio, documenti (funerali di Stato, processo, ricostruzione) [A]. DUPLICATO DELLA RIGA 14 (stessa entità) — da sciogliere (§8.4).</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>COLLAZIONE RETE 6.8.2026: stragi.it/archivio/documenti; nella Rete (memoria.cultura.gov.it). Archivio di Memoria del processo ai mandanti (RGNR 2/18) in digitalizzazione dal 2025, non ancora integralmente online — da riverificare.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
@@ -6299,13 +6334,21 @@
       <c r="G16" s="3" t="inlineStr"/>
       <c r="H16" s="3" t="inlineStr"/>
       <c r="I16" s="3" t="inlineStr"/>
-      <c r="J16" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K16" s="8" t="inlineStr"/>
-      <c r="L16" s="8" t="inlineStr"/>
+      <c r="J16" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Mappe di Memoria (mappedimemoria.it): archivio digitale sui luoghi delle stragi, del terrorismo e della violenza politica; Univ. di Bologna (Dip. Scienze dell'educazione), nella convenzione MIUR-associazioni delle vittime; copre Italicus 1974, Bologna 1980, Rapido 904 1984 [A].</t>
+        </is>
+      </c>
+      <c r="K16" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L16" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE RETE 6.8.2026: mappedimemoria.it, memoria.cultura.gov.it, UniBo. Ente confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
@@ -6341,13 +6384,21 @@
       <c r="G17" s="3" t="inlineStr"/>
       <c r="H17" s="3" t="inlineStr"/>
       <c r="I17" s="3" t="inlineStr"/>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K17" s="8" t="inlineStr"/>
-      <c r="L17" s="8" t="inlineStr"/>
+      <c r="J17" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — archivio900.it: portale di documentazione sul Novecento e sul terrorismo italiano e internazionale; libri, articoli, documenti e atti processuali; registro di 170 vittime del terrorismo 1967-2003 [A]. Risorsa documentale consultabile, non un archivio di Stato.</t>
+        </is>
+      </c>
+      <c r="K17" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L17" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: archivio900.it. Confermato come risorsa documentale.</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6433,13 +6484,21 @@
       <c r="G19" s="3" t="inlineStr"/>
       <c r="H19" s="3" t="inlineStr"/>
       <c r="I19" s="3" t="inlineStr"/>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr"/>
-      <c r="L19" s="8" t="inlineStr"/>
+      <c r="J19" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — l'Archivio di Stato di Milano conserva il fondo «Processo per la strage di piazza Fontana (Salvini)» (inventario a cura di F. Lisanti) e un distinto fondo «(Procura)» [A]. Istruttoria del giudice Salvini 1989-1997; sentenze istruttorie 18.3.1995 e 3.2.1998; fondo chiuso nel 2018.</t>
+        </is>
+      </c>
+      <c r="K19" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L19" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE RETE 6.8.2026: archiviodistatomilano.cultura.gov.it (inventari PDF), memoria.cultura.gov.it. Nome proprio disponibile: giudice Guido Salvini.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
@@ -6475,13 +6534,21 @@
       <c r="G20" s="3" t="inlineStr"/>
       <c r="H20" s="3" t="inlineStr"/>
       <c r="I20" s="3" t="inlineStr"/>
-      <c r="J20" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K20" s="8" t="inlineStr"/>
-      <c r="L20" s="8" t="inlineStr"/>
+      <c r="J20" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Archivio storico del Corriere della Sera, documentazione storico-giornalistica dal 1876 a oggi; numeri digitalizzati, prime pagine e articoli d'epoca consultabili online (archiviostorico.corriere.it) [A].</t>
+        </is>
+      </c>
+      <c r="K20" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L20" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: archiviostorico.corriere.it, cataloghi di ateneo. Ente confermato; utile per la datazione della ricezione.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
@@ -6521,13 +6588,21 @@
       </c>
       <c r="H21" s="3" t="inlineStr"/>
       <c r="I21" s="3" t="inlineStr"/>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr"/>
-      <c r="L21" s="8" t="inlineStr"/>
+      <c r="J21" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — ArchivioAntimafia (archivioantimafia.org): raccoglie e pubblica integralmente documenti su mafia e antimafia — sentenze e atti processuali in PDF, verbali, registrazioni [A] (es. atti Falcone/Capaci, trattativa Stato-mafia, Mafia Capitale).</t>
+        </is>
+      </c>
+      <c r="K21" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L21" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: archivioantimafia.org/sentenze.php, /testi.php. Testi integrali senza censura né sintesi — confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Blocco 2 (norme e istituzioni italiane) + chiusura parziali
Riscontro su Gazzetta Ufficiale/atti. 6 confermati (verde): L.124/2007 (segreto di
Stato, capo V), COPASIR (art.30 L.124/2007), L.82/2014 (Commissione Moro), art.53
c.16-ter d.lgs.165/2001 (pantouflage), L.17/1982 Anselmi (art.18 Cost./scioglimento
P2), direttive di desecretazione Prodi/Renzi (da integrare con Draghi 2021).
Parziali risolti: riga 11 fontitaliarepubblicana.it = ERRORE (dominio non risolve;
reale portale CNR portalefontirepubblicaitaliana.cnr.it, rosso); duplicazione 14=15
sciolta (riga 14 canonica confermata, riga 15 marcata duplicato da eliminare §8.4).
Nomi propri recuperati: Fioroni, Anselmi, Spadolini.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
+++ b/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
@@ -153,6 +153,9 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -6084,19 +6087,19 @@
       <c r="G11" s="3" t="inlineStr"/>
       <c r="H11" s="3" t="inlineStr"/>
       <c r="I11" s="3" t="inlineStr"/>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>PARZIALE — l'ente esiste (Portale delle fonti per la storia della Repubblica italiana, infrastruttura del CNR, accesso unico a fonti dal 1946 [A]), ma il DOMINIO va accertato: le fonti danno il portale come portalefontirepubblicaitaliana.cnr.it, non fontitaliarepubblicana.it [B]. Da confermare che il dominio del repertorio risolva o rediriga.</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
+      <c r="J11" s="17" t="inlineStr">
+        <is>
+          <t>ERRORE (dominio) — fontitaliarepubblicana.it NON risolve (ENOTFOUND) e nessuna fonte lo cita; l'ente reale è il «Portale delle fonti per la storia della Repubblica italiana» del CNR, a portalefontirepubblicaitaliana.cnr.it [B]. CORREZIONE: sostituire il dominio. Limite: DNS verificato dall'ambiente, da confermare sull'originale.</t>
+        </is>
+      </c>
+      <c r="K11" s="17" t="inlineStr">
         <is>
           <t>6.8.2026</t>
         </is>
       </c>
-      <c r="L11" s="8" t="inlineStr">
-        <is>
-          <t>COLLAZIONE RETE 6.8.2026: portalefontirepubblicaitaliana.cnr.it (CNR), Istituto Sturzo, storiadigitale.it; collegato al Centro Flamigni. DOMINIO DA RISCONTRARE.</t>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: dominio non risolve; CNR (portalefontirepubblicaitaliana.cnr.it), Istituto Sturzo, storiadigitale.it. DOMINIO DA CORREGGERE.</t>
         </is>
       </c>
     </row>
@@ -6234,19 +6237,19 @@
       <c r="G14" s="3" t="inlineStr"/>
       <c r="H14" s="3" t="inlineStr"/>
       <c r="I14" s="3" t="inlineStr"/>
-      <c r="J14" s="8" t="inlineStr">
-        <is>
-          <t>CONFERMATO come ente, MA DUPLICATO DELLA RIGA 15: l'Associazione familiari delle vittime della strage di Bologna del 2.8.1980 È il soggetto titolare di stragi.it (riga 15) [A]. Duplicazione fra voci da sciogliere (§8.4); tenuta in sospeso finché non si decide quale conservare e fondere.</t>
-        </is>
-      </c>
-      <c r="K14" s="8" t="inlineStr">
+      <c r="J14" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO (voce canonica della coppia duplicata 14/15) — Associazione tra i familiari delle vittime della strage di Bologna del 2.8.1980, soggetto conservatore; sito stragi.it, archivio consultabile di foto/video/audio/documenti [A]. La riga 15 (stragi.it) ne è la sola istanza web: da eliminare come duplicato (§8.4).</t>
+        </is>
+      </c>
+      <c r="K14" s="16" t="inlineStr">
         <is>
           <t>6.8.2026</t>
         </is>
       </c>
-      <c r="L14" s="8" t="inlineStr">
-        <is>
-          <t>COLLAZIONE 6.8.2026: stragi.it, memoria.cultura.gov.it. STESSA ENTITÀ della riga 15.</t>
+      <c r="L14" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE RETE 6.8.2026: stragi.it, memoria.cultura.gov.it. Voce canonica; assorbe la riga 15.</t>
         </is>
       </c>
     </row>
@@ -6284,19 +6287,19 @@
       <c r="G15" s="3" t="inlineStr"/>
       <c r="H15" s="3" t="inlineStr"/>
       <c r="I15" s="3" t="inlineStr"/>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>CONFERMATO — stragi.it è il sito dell'Associazione familiari vittime strage Bologna 2.8.1980; archivio consultabile di foto, video, audio, documenti (funerali di Stato, processo, ricostruzione) [A]. DUPLICATO DELLA RIGA 14 (stessa entità) — da sciogliere (§8.4).</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr">
+      <c r="J15" s="17" t="inlineStr">
+        <is>
+          <t>DUPLICATO DELLA RIGA 14 — stragi.it è il sito dell'Associazione familiari vittime strage Bologna (riga 14, canonica). Voce da eliminare nel passo §8.4; il contenuto è conservato sulla riga 14 [A].</t>
+        </is>
+      </c>
+      <c r="K15" s="17" t="inlineStr">
         <is>
           <t>6.8.2026</t>
         </is>
       </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>COLLAZIONE RETE 6.8.2026: stragi.it/archivio/documenti; nella Rete (memoria.cultura.gov.it). Archivio di Memoria del processo ai mandanti (RGNR 2/18) in digitalizzazione dal 2025, non ancora integralmente online — da riverificare.</t>
+      <c r="L15" s="17" t="inlineStr">
+        <is>
+          <t>Duplicato di riga 14 (§8.4). Contenuto conservato sulla canonica.</t>
         </is>
       </c>
     </row>
@@ -8842,13 +8845,21 @@
         </is>
       </c>
       <c r="I66" s="3" t="inlineStr"/>
-      <c r="J66" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K66" s="8" t="inlineStr"/>
-      <c r="L66" s="8" t="inlineStr"/>
+      <c r="J66" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO e integrato — desecretazione/versamento all'Archivio Centrale dello Stato per direttiva: Prodi (DPCM 8.4.2008), Renzi (22.4.2014) e — DA AGGIUNGERE — Draghi (2021, su Gladio e Loggia P2). Versamenti dal 1.8.2014; ~77 versamenti, 156 uffici, ~2.000 buste [A]. OMESSO E DISPONIBILE: la direttiva Draghi 2021.</t>
+        </is>
+      </c>
+      <c r="K66" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L66" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: acs.cultura.gov.it (Direttiva Renzi/Guida ai fondi STRAGI), archivi.cultura.gov.it. Confermato; integrare Draghi 2021.</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8892,13 +8903,21 @@
         </is>
       </c>
       <c r="I67" s="3" t="inlineStr"/>
-      <c r="J67" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K67" s="8" t="inlineStr"/>
-      <c r="L67" s="8" t="inlineStr"/>
+      <c r="J67" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Legge 3 agosto 2007 n.124, «Sistema di informazione per la sicurezza della Repubblica e nuova disciplina del segreto», pubblicata in G.U. n.187 del 13.8.2007; il capo V disciplina la tutela del segreto di Stato [A].</t>
+        </is>
+      </c>
+      <c r="K67" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L67" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: gazzettaufficiale.it, sicurezzanazionale.gov.it, Camera. Norma confermata.</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -8942,13 +8961,21 @@
         </is>
       </c>
       <c r="I68" s="3" t="inlineStr"/>
-      <c r="J68" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K68" s="8" t="inlineStr"/>
-      <c r="L68" s="8" t="inlineStr"/>
+      <c r="J68" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Comitato parlamentare per la sicurezza della Repubblica (COPASIR), istituito dall'art.30 della L.124/2007; 5 deputati + 5 senatori, sede a Palazzo San Macuto [A] (riscontro sull'atto istitutivo).</t>
+        </is>
+      </c>
+      <c r="K68" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L68" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: L.124/2007 (atto istitutivo), parlamento.it. Organo confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8992,13 +9019,21 @@
         </is>
       </c>
       <c r="I69" s="3" t="inlineStr"/>
-      <c r="J69" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K69" s="8" t="inlineStr"/>
-      <c r="L69" s="8" t="inlineStr"/>
+      <c r="J69" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Legge 30 maggio 2014 n.82: istituisce la Commissione parlamentare d'inchiesta sul rapimento e sulla morte di Aldo Moro; G.U. n.125 del 31.5.2014; Commissione costituita il 2.10.2014, presidente Giuseppe Fioroni; termine prorogato a fine XVII legislatura (DL 210/2015 conv. L.21/2016) [A]. NOME DISPONIBILE: Giuseppe Fioroni.</t>
+        </is>
+      </c>
+      <c r="K69" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L69" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: gazzettaufficiale.it, inchieste.camera.it/moro, parlamento.it. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -9042,13 +9077,21 @@
         </is>
       </c>
       <c r="I70" s="3" t="inlineStr"/>
-      <c r="J70" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K70" s="8" t="inlineStr"/>
-      <c r="L70" s="8" t="inlineStr"/>
+      <c r="J70" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — divieto di «pantouflage», art.53 comma 16-ter del d.lgs. 165/2001 (TUPI): il dipendente che ha esercitato poteri autoritativi/negoziali non può, per 3 anni dalla cessazione, lavorare presso i privati destinatari di quei poteri; sanzione di nullità; linee guida ANAC [A].</t>
+        </is>
+      </c>
+      <c r="K70" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L70" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: anticorruzione.it (linee guida pantouflage), Altalex, Diritto.it. Norma confermata.</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -9192,13 +9235,21 @@
         </is>
       </c>
       <c r="I73" s="3" t="inlineStr"/>
-      <c r="J73" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K73" s="8" t="inlineStr"/>
-      <c r="L73" s="8" t="inlineStr"/>
+      <c r="J73" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Legge 25 gennaio 1982 n.17 (Anselmi/Spadolini), norme di attuazione dell'art.18 Cost. in materia di associazioni segrete e scioglimento della Loggia P2; G.U. del 28.1.1982; governo Spadolini I [A]. NOMI DISPONIBILI: Tina Anselmi, Giovanni Spadolini.</t>
+        </is>
+      </c>
+      <c r="K73" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L73" s="16" t="inlineStr">
+        <is>
+          <t>COLLAZIONE 6.8.2026: gazzettaufficiale.it (082U0017), Wikipedia/Legge Anselmi, vLex. Norma confermata.</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Blocco 2 completa il fronte italiano: 7 atti/relazioni verificati
Riscontro esterno: Relazione COPASIR 2021-2022 (feb-ago 2022, pres. Urso),
CEDU Grande Oriente d'Italia c. Italia ric. 29550/17 (art.8; Grande Camera 7.7.2026),
Commissione antimafia sulla massoneria Doc. XXIII n.33 (rel. Bindi), operazioni
Kyterion e Grimilde (cosca Grande Aracri), processo P3 (sent. 16.3.2018). Processo
Gotha parziale (giallo): primo grado confermato, esito d'appello 2026 da riscontrare;
aggiungere l'inchiesta Alchimia. Foglio 01: 44/82 verificate. Fronte italiano completo
(22 voci: 20 confermate, 2 difetti). Aggiornate sezioni 7 e 8 del CLAUDE.md con i nomi
propri recuperati.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
+++ b/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
@@ -9135,13 +9135,21 @@
         </is>
       </c>
       <c r="I71" s="3" t="inlineStr"/>
-      <c r="J71" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K71" s="8" t="inlineStr"/>
-      <c r="L71" s="8" t="inlineStr"/>
+      <c r="J71" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Relazione annuale del COPASIR 2021-2022 (attività febbraio-agosto 2022), trasmessa al Parlamento a inizio agosto 2022, anticipata per lo scioglimento delle Camere; presidente Adolfo Urso. Ravvisa «una sostanziale debolezza degli interventi» contro disinformazione e interferenze (infowarfare russa/cinese, golden power) [A]. NOME DISPONIBILE: Adolfo Urso.</t>
+        </is>
+      </c>
+      <c r="K71" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L71" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Formiche, Askanews, PublicPolicy (PDF). Confermato; due indagini incompiute coerenti col contesto.</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9293,13 +9301,21 @@
         </is>
       </c>
       <c r="I74" s="3" t="inlineStr"/>
-      <c r="J74" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K74" s="8" t="inlineStr"/>
-      <c r="L74" s="8" t="inlineStr"/>
+      <c r="J74" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — CEDU, Grande Oriente d'Italia c. Italia, ric. 29550/17: violazione dell'art.8 per la perquisizione e il sequestro (2017) di 39 faldoni di schede degli iscritti alle logge di Sicilia e Calabria disposti dalla Commissione antimafia [A]. Sentenza di camera 19.12.2024; la GRANDE CAMERA il 7.7.2026 ha respinto l'appello del governo — DA AGGIUNGERE.</t>
+        </is>
+      </c>
+      <c r="K74" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L74" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: giustizia.it (sentenze CEDU), Federprivacy, Rivista Penale. Integrare la Grande Camera 7.7.2026.</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9343,13 +9359,21 @@
         </is>
       </c>
       <c r="I75" s="3" t="inlineStr"/>
-      <c r="J75" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K75" s="8" t="inlineStr"/>
-      <c r="L75" s="8" t="inlineStr"/>
+      <c r="J75" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Commissione parlamentare antimafia (XVII leg.), relazione sulle infiltrazioni di Cosa Nostra e 'ndrangheta nella massoneria (Sicilia e Calabria), Doc. XXIII n.33, approvata il 21.12.2017; relatrice Rosy Bindi. Castelvetrano: loggia Francisco Ferrer, tre assessori massoni (due iscritti al GOI) [A]. NOME DISPONIBILE: Rosy Bindi.</t>
+        </is>
+      </c>
+      <c r="K75" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L75" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: inchieste.camera.it/mafie, Avviso Pubblico, Editoriale Domani. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -9395,11 +9419,19 @@
       <c r="I76" s="3" t="inlineStr"/>
       <c r="J76" s="8" t="inlineStr">
         <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K76" s="8" t="inlineStr"/>
-      <c r="L76" s="8" t="inlineStr"/>
+          <t>PARZIALE — processo Gotha (Reggio Calabria), dalla fusione di Mammasantissima, Reghion, Fata Morgana, Sistema Reggio e — DA AGGIUNGERE — Alchimia (cinque inchieste, non quattro). Rito abbreviato: primo grado marzo 2018, giudice Pasquale Laganà, 28 condanne e 10 assoluzioni; motivazioni nov. 2018 [A]. L'ESITO D'APPELLO DEL MAGGIO 2026 (azzeramento delle condanne sulla componente riservata) NON riscontrato dalle fonti consultate — da verificare [C]. NOME DISPONIBILE: Pasquale Laganà.</t>
+        </is>
+      </c>
+      <c r="K76" s="8" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L76" s="8" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Wikipedia/Processo Gotha, Il Fatto (motivazioni), citynow. Primo grado confermato; appello 2026 da riscontrare; aggiungere Alchimia.</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -9439,13 +9471,21 @@
       </c>
       <c r="H77" s="3" t="inlineStr"/>
       <c r="I77" s="3" t="inlineStr"/>
-      <c r="J77" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K77" s="8" t="inlineStr"/>
-      <c r="L77" s="8" t="inlineStr"/>
+      <c r="J77" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — operazione Kyterion, DDA di Catanzaro: 29.1.2015, 37 fermati della cosca Grande Aracri (Cutro/Crotonese); Kyterion 2 il 4.1.2016, 16 arresti, con tentativi di aggancio a Vaticano, Cassazione e ambienti massonici attribuiti a Nicolino Grande Aracri [A]. NOMI DISPONIBILI: Nicolino ed Ernesto Grande Aracri (ergastolo per l'omicidio Dragone, confermato in Cassazione 4.6.2019).</t>
+        </is>
+      </c>
+      <c r="K77" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L77" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Gazzetta del Sud, Zoom24, Reggio Report. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -9535,13 +9575,21 @@
         </is>
       </c>
       <c r="I79" s="3" t="inlineStr"/>
-      <c r="J79" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K79" s="8" t="inlineStr"/>
-      <c r="L79" s="8" t="inlineStr"/>
+      <c r="J79" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — operazione/processo Grimilde, DDA di Bologna: maggio 2019, poi 25.6.2019, 16 arresti; ramo emiliano (Reggio Emilia-Parma-Piacenza) della cosca Grande Aracri. Condanna definitiva a oltre 12 anni dell'esponente politico Giuseppe Caruso (ex presidente del consiglio comunale di Piacenza, FdI); in appello a Bologna 24 condanne, pena max 19a6m a Francesco Grande Aracri [A]. NOMI DISPONIBILI: Giuseppe Caruso, Francesco Grande Aracri.</t>
+        </is>
+      </c>
+      <c r="K79" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L79" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Quotidiano del Sud, La Via Libera, il Resto del Carlino. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9585,13 +9633,21 @@
         </is>
       </c>
       <c r="I80" s="3" t="inlineStr"/>
-      <c r="J80" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K80" s="8" t="inlineStr"/>
-      <c r="L80" s="8" t="inlineStr"/>
+      <c r="J80" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — processo P3, Tribunale di Roma IX sez. penale, sentenza 16.3.2018: la P3 è ritenuta associazione segreta (violazione della legge Anselmi) volta a condizionare gli organi costituzionali. Flavio Carboni 6 anni e 6 mesi (già coinvolto nel crac del Banco Ambrosiano); Arcangelo Martino 4a9m; Denis Verdini assolto dall'accusa più grave, 1a3m per finanziamento illecito; prescrizione per Ugo Cappellacci (ex presidente Regione Sardegna, abuso d'ufficio) [A]. NOMI: Carboni, Martino, Verdini, Cappellacci.</t>
+        </is>
+      </c>
+      <c r="K80" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L80" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: ANSA, Radio Radicale (sentenza), Unione Sarda, Today. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Blocco esteri 1 (Germania): 8 archivi confermati
Riscontro esterno: Commissione storici del BND (UHK 2011), distruzione atti BfV
"Aktion Konfetti"/NSU-Rennsteig (11.11.2011), atti LfV Hessen segretati 120 anni
(Yozgat/Temme), Bund Deutscher Jugend/Technischer Dienst (stay-behind, CIA, Odenwald),
schedario Rosenholz della HVA (BStU, 2003-2004), PKGr del Bundestag (1956-2009, art.45d
GG), commissioni sulle continuita naziste (Das Amt/Rosenburg), procedimento Oktoberfest
1980 (Kohler, riaperto 2014/archiviato 2020). Tutti verde. Foglio 01: 52/82. Nomi propri
recuperati (Dulffer, Krieger, Temme, Barbie, Adenauer, Gortemaker, Kohler, Chaussy, ecc.).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019coNthnDEGPwsM4yiT7gT7
</commit_message>
<xml_diff>
--- a/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
+++ b/repertorio/ITALIA_NERA_REPERTORIO_RIPARATO_E_FOGLIO_DI_VERIFICA2.xlsx
@@ -7361,13 +7361,21 @@
       </c>
       <c r="H36" s="3" t="inlineStr"/>
       <c r="I36" s="3" t="inlineStr"/>
-      <c r="J36" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K36" s="8" t="inlineStr"/>
-      <c r="L36" s="8" t="inlineStr"/>
+      <c r="J36" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Commissione indipendente di storici sul BND (UHK), istituita nel 2011 dallo stesso BND per la storia del servizio e della Gehlen-Org 1945-1968; ~2,4 mln€ dal bilancio del BND; 11 volumi pubblicati [A]. NOMI: Jost Dülffer, Klaus-Dietmar Henke, Wolfgang Krieger, Rolf-Dieter Müller.</t>
+        </is>
+      </c>
+      <c r="K36" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L36" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Bundestag (hib), Uni Marburg, Clio-online, Wikipedia BND. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7407,13 +7415,21 @@
       </c>
       <c r="H37" s="3" t="inlineStr"/>
       <c r="I37" s="3" t="inlineStr"/>
-      <c r="J37" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K37" s="8" t="inlineStr"/>
-      <c r="L37" s="8" t="inlineStr"/>
+      <c r="J37" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Ufficio federale per la protezione della Costituzione (BfV): l'11.11.2011, stesso giorno dell'avvio delle indagini della Procura federale sull'NSU, un capodivisione ordinò la distruzione di fascicoli («Aktion Konfetti») su 7 informatori (V-Leute) dell'«Operation Rennsteig» (1997-2003, scena neonazista in Turingia) [A]. NSU: Mundlos, Böhnhardt, Zschäpe.</t>
+        </is>
+      </c>
+      <c r="K37" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L37" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Tagesspiegel, taz, Verfassungsblog. Accertato da Procura federale e commissione d'inchiesta del Bundestag.</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7453,13 +7469,21 @@
       </c>
       <c r="H38" s="3" t="inlineStr"/>
       <c r="I38" s="3" t="inlineStr"/>
-      <c r="J38" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K38" s="8" t="inlineStr"/>
-      <c r="L38" s="8" t="inlineStr"/>
+      <c r="J38" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Ufficio regionale dell'Assia per la protezione della Costituzione (LfV Hessen): rapporto interno di revisione degli atti (nov. 2014) sull'omicidio NSU di Kassel (Halit Yozgat) e sul funzionario Andreas Temme, presente sulla scena; segretato per 120 anni («nessun caso comparabile»), poi ridotto a 30 [A]. NOMI: Andreas Temme, Halit Yozgat.</t>
+        </is>
+      </c>
+      <c r="K38" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L38" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Wikipedia/Halit Yozgat, Telepolis/Heise, t-online, NSU-Watch. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7503,13 +7527,21 @@
         </is>
       </c>
       <c r="I39" s="3" t="inlineStr"/>
-      <c r="J39" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K39" s="8" t="inlineStr"/>
-      <c r="L39" s="8" t="inlineStr"/>
+      <c r="J39" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Bund Deutscher Jugend (BDJ) e il suo «Technischer Dienst», rete stay-behind: fondata nel giugno 1950 su iniziativa della CIA (OPC), sciolta a fine 1952/inizio 1953; deposito d'armi nell'Odenwald (Waldmichelbach); liste di ~40 dirigenti SPD/KPD da eliminare; scoperta dopo la denuncia di Hans Otto alla polizia di Francoforte (9.9.1952) [A]. NOMI: Hans Otto, Klaus Barbie.</t>
+        </is>
+      </c>
+      <c r="K39" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L39" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Wikipedia (en/de) BDJ, Lecorte, Vorwärts. Confermato; finanziamento USA ~50.000$/mese.</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7553,13 +7585,21 @@
         </is>
       </c>
       <c r="I40" s="3" t="inlineStr"/>
-      <c r="J40" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K40" s="8" t="inlineStr"/>
-      <c r="L40" s="8" t="inlineStr"/>
+      <c r="J40" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — schedario microfilmato «Rosenholz» della HVA (spionaggio estero della Stasi/DDR): 381 supporti ottici, ~280.000 file (il repertorio dice ~293.000 — SCARTO MINORE da verificare); desecretato il 26.6.2003, consultabile presso il BStU/Bundesarchiv dal marzo 2004 [A]. Cerniera: ~90% delle persone schedate non erano IM.</t>
+        </is>
+      </c>
+      <c r="K40" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L40" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Bundesarchiv (Rosenholz), Wikipedia (de/en). Confermato; scarto sul numero di schede.</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7599,13 +7639,21 @@
       </c>
       <c r="H41" s="3" t="inlineStr"/>
       <c r="I41" s="3" t="inlineStr"/>
-      <c r="J41" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="inlineStr"/>
-      <c r="L41" s="8" t="inlineStr"/>
+      <c r="J41" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — Organo parlamentare di controllo sui servizi (PKGr), Bundestag: 1956 comitato di fiduciari (PMVG, Adenauer, senza base legale, solo BND fino al 1964); 1978 base legislativa (PKK); 1999 rinominato PKGr; 2009 ancoraggio costituzionale nell'art.45d GG; controlla BND, BfV e MAD [A]. NOME: Konrad Adenauer.</t>
+        </is>
+      </c>
+      <c r="K41" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L41" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Bundestag (einführung), Wikipedia PKGr, art.45d GG, PKGrG. Confermato.</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7645,13 +7693,21 @@
       </c>
       <c r="H42" s="3" t="inlineStr"/>
       <c r="I42" s="3" t="inlineStr"/>
-      <c r="J42" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K42" s="8" t="inlineStr"/>
-      <c r="L42" s="8" t="inlineStr"/>
+      <c r="J42" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — serie di commissioni indipendenti sulle continuità istituzionali dopo il 1945: ministero degli Esteri (2005 → «Das Amt», 2010), ministero delle Finanze (2009, sul Reichsfinanzministerium), ministero della Giustizia (2012 → «Die Akte Rosenburg») [A]. NOMI: Manfred Görtemaker, Christoph Safferling.</t>
+        </is>
+      </c>
+      <c r="K42" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L42" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Siscalt, diplo.de, ANRP. Confermato; fenomeno sistemico.</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -9691,13 +9747,21 @@
         </is>
       </c>
       <c r="I81" s="3" t="inlineStr"/>
-      <c r="J81" s="8" t="inlineStr">
-        <is>
-          <t>da riverificare</t>
-        </is>
-      </c>
-      <c r="K81" s="8" t="inlineStr"/>
-      <c r="L81" s="8" t="inlineStr"/>
+      <c r="J81" s="16" t="inlineStr">
+        <is>
+          <t>CONFERMATO — procedimento tedesco sull'attentato dell'Oktoberfest (Monaco, 26.9.1980): 12 vittime più l'attentatore Gundolf Köhler, 200+ feriti; tesi iniziale del singolo; indagini della Procura federale riaperte a fine 2014 (grazie a Ulrich Chaussy e all'avv. Werner Dietrich), archiviate nel luglio 2020 riconoscendo il movente politico di estrema destra [A]. Pubblicazione online dei documenti da parte del Bundesarchiv NON riscontrata — da verificare. NOMI: Gundolf Köhler, Ulrich Chaussy, Werner Dietrich.</t>
+        </is>
+      </c>
+      <c r="K81" s="16" t="inlineStr">
+        <is>
+          <t>6.8.2026</t>
+        </is>
+      </c>
+      <c r="L81" s="16" t="inlineStr">
+        <is>
+          <t>RISCONTRO 6.8.2026: Wikipedia/Oktoberfest bombing, WSWS, openDemocracy. Confermato; pubblicazione Bundesarchiv da riscontrare.</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">

</xml_diff>